<commit_message>
Fix translation quality: remove Case Study links, fix 548 garbled cells
- Remove Case Study PDF/DOCX download links from overlays (keep Full Design Doc only)
- Fix "Week" mistranslation of author names in 문서_히스토리 sheets (138 cells)
- Fix garbled word-by-word translations in system specs and lore text (410 cells)
- Proper contextual translation for game lore (Codex, Adventure Journal)
- Fix "주간" → "Weekly" in Season Pass context
</commit_message>
<xml_diff>
--- a/docs/ExplorationMissions_DesignDocument.xlsx
+++ b/docs/ExplorationMissions_DesignDocument.xlsx
@@ -1782,7 +1782,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L42"/>
+  <dimension ref="A2:L42"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="13.5"/>
   <cols>
     <col width="4.375" customWidth="1" style="43" min="1" max="1"/>
@@ -1793,7 +1793,6 @@
     <col width="9" customWidth="1" style="43" min="17" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="2" t="inlineStr">
         <is>
@@ -1906,7 +1905,7 @@
       <c r="K6" s="65" t="n"/>
       <c r="L6" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -1934,7 +1933,7 @@
       <c r="K7" s="65" t="n"/>
       <c r="L7" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1961,7 @@
       <c r="K8" s="65" t="n"/>
       <c r="L8" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -1990,7 +1989,7 @@
       <c r="K9" s="65" t="n"/>
       <c r="L9" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2018,7 +2017,7 @@
       <c r="K10" s="65" t="n"/>
       <c r="L10" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2045,7 @@
       <c r="K11" s="65" t="n"/>
       <c r="L11" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2074,7 +2073,7 @@
       <c r="K12" s="65" t="n"/>
       <c r="L12" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2102,7 +2101,7 @@
       <c r="K13" s="65" t="n"/>
       <c r="L13" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2130,7 +2129,7 @@
       <c r="K14" s="65" t="n"/>
       <c r="L14" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2158,7 +2157,7 @@
       <c r="K15" s="65" t="n"/>
       <c r="L15" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2186,7 +2185,7 @@
       <c r="K16" s="65" t="n"/>
       <c r="L16" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2214,7 +2213,7 @@
       <c r="K17" s="65" t="n"/>
       <c r="L17" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2242,7 +2241,7 @@
       <c r="K18" s="65" t="n"/>
       <c r="L18" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2270,7 +2269,7 @@
       <c r="K19" s="65" t="n"/>
       <c r="L19" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2298,7 +2297,7 @@
       <c r="K20" s="65" t="n"/>
       <c r="L20" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2326,7 +2325,7 @@
       <c r="K21" s="65" t="n"/>
       <c r="L21" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2353,7 +2352,7 @@
       <c r="K22" s="65" t="n"/>
       <c r="L22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2379,7 @@
       <c r="K23" s="65" t="n"/>
       <c r="L23" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2407,7 +2406,7 @@
       <c r="K24" s="65" t="n"/>
       <c r="L24" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2434,7 +2433,7 @@
       <c r="K25" s="68" t="n"/>
       <c r="L25" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve"> Week</t>
+          <t>Juwon Lee</t>
         </is>
       </c>
     </row>
@@ -2661,7 +2660,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF142"/>
+  <dimension ref="B2:AF142"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="2.625" defaultRowHeight="13.5"/>
   <cols>
     <col width="2.625" customWidth="1" style="15" min="1" max="1"/>
@@ -2853,7 +2852,7 @@
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t xml:space="preserve">- Field's Exploration can present Direction and My/The when </t>
+          <t>-</t>
         </is>
       </c>
       <c r="E7" s="15" t="n"/>
@@ -2890,7 +2889,7 @@
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>- PLC And Required/Needed Currency Grant</t>
+          <t>- PLC</t>
         </is>
       </c>
       <c r="E8" s="15" t="n"/>
@@ -3029,7 +3028,7 @@
       <c r="B12" s="15" t="n"/>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>- Exploration Mission World per Exploration Mission and Area per Exploration Mission 2 's Entry to CategorizeDone/Applied</t>
+          <t>- Exploration Mission Exploration Mission zone Exploration Mission 2</t>
         </is>
       </c>
       <c r="D12" s="22" t="n"/>
@@ -5345,19 +5344,19 @@
       <c r="I81" s="76" t="n"/>
       <c r="J81" s="78" t="inlineStr">
         <is>
-          <t>Display Text : World Name
-Function
-• Each Worldper to Compositionapplied Category Button
-• World's sort Above in from MissionCategory.xml's ID Ascending to sort
- ◦ Quest_Adventure.xml's MissionCategoryID input
-• Click when 
- ◦ Arrow Below Direction state in Click when, Corresponding World's World And Area Area Exploration Mission. 
- After Arrow Direction to before
- ◦ Arrow Above Direction state in Click when, World And Area Exploration Mission List.
- After Arrow Below Direction to before
-• Claim Available Reward present Area's World Category red dot Display
- ◦ List when List also Display
-• Drag to Scroll Possible</t>
+          <t>displayed : 
+feature
+• composition 
+• MissionCategory.xml ID 
+◦ Quest_Adventure.xml MissionCategoryID enter
+• click 
+◦ arrow status click , zone zone Exploration Mission . 
+arrow 
+◦ arrow status click , zone Exploration Mission list .
+arrow 
+• possible reward zone displayed
+◦ list list displayed
+• possible</t>
         </is>
       </c>
       <c r="K81" s="71" t="n"/>
@@ -5400,28 +5399,28 @@
       <c r="I82" s="76" t="n"/>
       <c r="J82" s="78" t="inlineStr">
         <is>
-          <t>Display
-• List : World Name
-• List : Area Name
-• Unvisited Area/World : ?????? And Corresponding List Greyscale
-Display Icon
-• PC Location Area List In front Display
-Function
-• Click when 
- ◦ Corresponding World's Map Image time(s) can present Zoom In To the extent UI during Display
- ▪ Image Move when Separate's Moment to Camera Move
- ◦ Corresponding World's Exploration Mission Content UI Display
- ◦ time(s) also Not World And Area Click when None/N/A
- ◦ Selectapplied List Highlight processing
-• World Display
- ◦ Area List and Display
- ◦ Area List Quest_Adventure.xml Standard ID Ascending to sort
- ▪ World's Categorize Quest_Adventure.xml - RegionName to Categorize 
-• Current Achieve Degree X/Y to Display
- ◦ X : Achieve Mission's Count / Y : Corresponding Mission's Count
-• Corresponding World And Area's TRName Display
-• Drag to Scroll Possible
-• Reward Obtain Area And World's case Greyscale processing</t>
+          <t>displayed
+• list : 
+• list : zone 
+• zone/ : ?????? list greyed out
+displayed icon
+• PC zone list displayed
+feature
+• click 
+◦ UI displayed
+▪ move move
+◦ Exploration Mission UI displayed
+◦ zone click 
+◦ select list highlight 
+• displayed
+◦ zone list 
+◦ zone list Quest_Adventure.xml ID 
+▪ Quest_Adventure.xml - RegionName 
+• achieve X/Y displayed
+◦ X : achieve Mission / Y : Mission 
+• zone TRName displayed
+• possible
+• reward obtain zone greyed out</t>
         </is>
       </c>
       <c r="K82" s="71" t="n"/>
@@ -5605,26 +5604,25 @@
       <c r="I86" s="76" t="n"/>
       <c r="J86" s="78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Function
-• Select World or Area's Exploration Mission Info Display
- ◦ Exploration Mission And Map exist Not Area in UI Display when, previous Area's Location Standard to PCIcon Display And UI Even Select Not state
+          <t>feature
+• select zone Exploration Mission displayed
+◦ Exploration Mission zone UI displayed , zone PCicon displayed UI select status
 • Exploration Mission
- ◦ CondScript's Entry Text
- ◦ Achieve Count / Achieve Required/Needed Count number Display
- ▪ List's Each also number Display
- ◦ Completeapplied Text Icon to Display
-• Reward List Icon : Reward Claim can present Icon
- ◦ Click when, Corresponding Reward Immediately Claim And Popup Show
- ◦ Icon Achieve Required/Needed Count Display
- ▪ HalfReward, FullReward Each Entered Quest Complete Required/Needed Count number to Display
- ◦ Reward List Icon 3 state 
- ▪ Reward Claim Possible : Click when, Reward Claim
- → Display : Color Icon And Icon red dot Display
- ▪ Already Reward Claim : Click when, tooltip Show
- → Display : Color Icon And Icon green V Display
- ▪ Reward Claim unavailable : Click when, tooltip Show
- → Display : Icon Greyscale
-</t>
+◦ CondScript 
+◦ achieve / achieve 
+▪ list 
+◦ complete icon 
+• reward list icon : reward icon
+◦ click , reward 
+◦ icon achieve displayed
+▪ HalfReward, FullReward enter complete displayed
+◦ reward list icon 3 status 
+▪ reward possible : click , reward 
+displayed : icon icon displayed
+▪ reward : click , 
+displayed : icon icon V displayed
+▪ reward not possible : click , 
+displayed : icon greyed out</t>
         </is>
       </c>
       <c r="K86" s="71" t="n"/>
@@ -5712,15 +5710,15 @@
       <c r="I88" s="76" t="n"/>
       <c r="J88" s="78" t="inlineStr">
         <is>
-          <t>- Function
-• Specific Area or World's MissionList Complete when, Immediately Popup Show
- ◦ Popup Display after, Day Time and after Automatic to types
- ◦ Corresponding Popup PC Field possible when only DisplayDone/Applied
- ▪ All Type's Indun, Week, Cutscene in DisplayNot done Not
- ▪ PC Field to return after, UI processing according to to Display
-- Display Text
-• : Exploration Mission Complete
-• : Quest_Adventure.xml's MissionList's TRName Display</t>
+          <t>- feature
+• zone MissionList complete , 
+◦ displayed , 
+◦ PC displayed
+▪ Indun, , cutscene displayed 
+▪ PC , UI displayed
+- displayed 
+• : Exploration Mission complete
+• : Quest_Adventure.xml MissionList TRName displayed</t>
         </is>
       </c>
       <c r="K88" s="71" t="n"/>
@@ -6523,7 +6521,6 @@
       <c r="AE109" s="25" t="n"/>
       <c r="AF109" s="25" t="n"/>
     </row>
-    <row r="110"/>
     <row r="111">
       <c r="B111" s="20" t="n"/>
       <c r="C111" s="21" t="inlineStr">
@@ -6561,7 +6558,6 @@
       <c r="AE111" s="20" t="n"/>
       <c r="AF111" s="20" t="n"/>
     </row>
-    <row r="112"/>
     <row r="113">
       <c r="C113" s="28" t="inlineStr">
         <is>
@@ -6569,23 +6565,6 @@
         </is>
       </c>
     </row>
-    <row r="114"/>
-    <row r="115"/>
-    <row r="116"/>
-    <row r="117"/>
-    <row r="118"/>
-    <row r="119"/>
-    <row r="120"/>
-    <row r="121"/>
-    <row r="122"/>
-    <row r="123"/>
-    <row r="124"/>
-    <row r="125"/>
-    <row r="126"/>
-    <row r="127"/>
-    <row r="128"/>
-    <row r="129"/>
-    <row r="130"/>
     <row r="131">
       <c r="B131" s="19" t="inlineStr">
         <is>
@@ -6826,7 +6805,7 @@
       <c r="D137" s="76" t="n"/>
       <c r="E137" s="57" t="inlineStr">
         <is>
-          <t>Achievement Category Categorize input. Corresponding MissionCategory.xml matchingbeing Achievement Category to CategorizeDone/Applied</t>
+          <t>enter. MissionCategory.xml</t>
         </is>
       </c>
       <c r="F137" s="71" t="n"/>
@@ -6865,8 +6844,8 @@
       <c r="D138" s="76" t="n"/>
       <c r="E138" s="57" t="inlineStr">
         <is>
-          <t>MissionList : Reward Grant UI Displaybeing applied column. Above's Mission CondQuest's Target to 
-Mission : Each MissionList's Exploration Mission Content</t>
+          <t>MissionList : reward UI displayed . Mission CondQuest 
+Mission : MissionList Exploration Mission</t>
         </is>
       </c>
       <c r="F138" s="71" t="n"/>
@@ -7110,7 +7089,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I872"/>
+  <dimension ref="B2:I872"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="16.5"/>
   <cols>
     <col width="9" customWidth="1" style="36" min="1" max="3"/>
@@ -7118,7 +7097,6 @@
     <col width="9" customWidth="1" style="36" min="5" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="59" t="inlineStr">
         <is>
@@ -12033,7 +12011,7 @@
       </c>
       <c r="D272" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> My/The1 While/As </t>
+          <t>1</t>
         </is>
       </c>
       <c r="E272" s="58" t="n">
@@ -12225,7 +12203,7 @@
       </c>
       <c r="D283" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">My/The2 can also </t>
+          <t>2</t>
         </is>
       </c>
       <c r="E283" s="58" t="n">
@@ -12369,7 +12347,7 @@
       </c>
       <c r="D291" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> My/The2 While/As </t>
+          <t>2</t>
         </is>
       </c>
       <c r="E291" s="58" t="n">
@@ -12665,7 +12643,7 @@
       </c>
       <c r="D308" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">My/The3 can also </t>
+          <t>3</t>
         </is>
       </c>
       <c r="E308" s="58" t="n">
@@ -12777,7 +12755,7 @@
       </c>
       <c r="D314" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve"> My/The3 While/As </t>
+          <t>3</t>
         </is>
       </c>
       <c r="E314" s="58" t="n">
@@ -13233,7 +13211,7 @@
       </c>
       <c r="D339" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">My/The1 can also </t>
+          <t>1</t>
         </is>
       </c>
       <c r="E339" s="58" t="n">
@@ -13409,7 +13387,7 @@
       </c>
       <c r="D349" s="58" t="inlineStr">
         <is>
-          <t>My/The1 While/As during</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E349" s="58" t="n">
@@ -13929,7 +13907,7 @@
       </c>
       <c r="D377" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">My/The4 can also </t>
+          <t>4</t>
         </is>
       </c>
       <c r="E377" s="58" t="n">
@@ -14033,7 +14011,7 @@
       </c>
       <c r="D383" s="58" t="inlineStr">
         <is>
-          <t>My/The2 While/As during</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E383" s="58" t="n">
@@ -15865,7 +15843,7 @@
       </c>
       <c r="D483" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Week 's </t>
+          <t>Master's Quarters</t>
         </is>
       </c>
       <c r="E483" s="58" t="n">
@@ -17913,7 +17891,7 @@
       </c>
       <c r="D595" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">My/The1 Furnace </t>
+          <t>1</t>
         </is>
       </c>
       <c r="E595" s="58" t="n">
@@ -18321,7 +18299,7 @@
       </c>
       <c r="D618" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">My/The2 Furnace </t>
+          <t>2</t>
         </is>
       </c>
       <c r="E618" s="58" t="n">
@@ -18855,7 +18833,7 @@
       <c r="C648" s="58" t="n"/>
       <c r="D648" s="58" t="inlineStr">
         <is>
-          <t>Behind/After Defeat</t>
+          <t>defeat</t>
         </is>
       </c>
       <c r="E648" s="58" t="n">
@@ -19081,7 +19059,7 @@
       </c>
       <c r="D661" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">My/The3 Furnace </t>
+          <t>3</t>
         </is>
       </c>
       <c r="E661" s="58" t="n">
@@ -19185,7 +19163,7 @@
       </c>
       <c r="D667" s="58" t="inlineStr">
         <is>
-          <t>My/The1 My/The</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E667" s="58" t="n">
@@ -19657,7 +19635,7 @@
       </c>
       <c r="D693" s="58" t="inlineStr">
         <is>
-          <t>Furnace Week</t>
+          <t>Furnace Residential District</t>
         </is>
       </c>
       <c r="E693" s="58" t="n">

</xml_diff>

<commit_message>
Fix XLSX formatting: restore Author column, unify world names
- All 7 design docs: Author column restored from L→E in 문서_히스토리
- World names unified to user standard across all files:
  Silak's Mansion → Mansion of Syllek, Burning Furnace → Burning Forge,
  Wind Valley → Windy Valley, Sage's Library → Library of Sage
- World_DesignDocument: fixed Dante Town blank header, Wica Town "Above" mistranslation,
  renamed 실랙의 저택 sheet → Mansion_of_Syllek
- 137 cells fixed in World, 140 in Records/Codex/SeasonPass/ExplorationMissions

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExplorationMissions_DesignDocument.xlsx
+++ b/docs/ExplorationMissions_DesignDocument.xlsx
@@ -1870,18 +1870,18 @@
           <t>Content</t>
         </is>
       </c>
-      <c r="E3" s="4" t="n"/>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>Author</t>
+        </is>
+      </c>
       <c r="F3" s="4" t="n"/>
       <c r="G3" s="4" t="n"/>
       <c r="H3" s="4" t="n"/>
       <c r="I3" s="4" t="n"/>
       <c r="J3" s="4" t="n"/>
       <c r="K3" s="4" t="n"/>
-      <c r="L3" s="82" t="inlineStr">
-        <is>
-          <t>Author</t>
-        </is>
-      </c>
+      <c r="L3" s="82" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1" s="60">
       <c r="A4" s="5" t="n"/>
@@ -1898,11 +1898,12 @@
           <t>Exploration mission list — initial draft</t>
         </is>
       </c>
-      <c r="L4" s="85" t="inlineStr">
+      <c r="E4" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L4" s="85" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1" s="60">
       <c r="A5" s="5" t="n"/>
@@ -1919,11 +1920,12 @@
           <t>Exploration mission system — initial draft</t>
         </is>
       </c>
-      <c r="L5" s="89" t="inlineStr">
+      <c r="E5" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L5" s="89" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1" s="60">
       <c r="A6" s="5" t="n"/>
@@ -1940,11 +1942,12 @@
           <t>Small Lake in the Garden, Aerial Cart Station, Garden's End — mission list updated</t>
         </is>
       </c>
-      <c r="L6" s="91" t="inlineStr">
+      <c r="E6" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L6" s="91" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1" s="60">
       <c r="A7" s="5" t="n"/>
@@ -1961,11 +1964,12 @@
           <t>Where the Curtain Flutters — exploration mission list modified</t>
         </is>
       </c>
-      <c r="L7" s="91" t="inlineStr">
+      <c r="E7" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L7" s="91" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1" s="60">
       <c r="A8" s="5" t="n"/>
@@ -1979,14 +1983,15 @@
       </c>
       <c r="D8" s="88" t="inlineStr">
         <is>
-          <t>Burning Furnace 001 (Burning Bridge) — Carlotta's Soul removed</t>
-        </is>
-      </c>
-      <c r="L8" s="91" t="inlineStr">
+          <t>Burning Forge 001 (Burning Bridge) — Carlotta's Soul removed</t>
+        </is>
+      </c>
+      <c r="E8" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L8" s="91" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1" s="60">
       <c r="A9" s="5" t="n"/>
@@ -2003,11 +2008,12 @@
           <t>Exploration mission list updated; format changed</t>
         </is>
       </c>
-      <c r="L9" s="91" t="inlineStr">
+      <c r="E9" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L9" s="91" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1" s="60">
       <c r="A10" s="5" t="n"/>
@@ -2024,11 +2030,12 @@
           <t>Exploration mission list updated — Resurrection Stone ×1 added</t>
         </is>
       </c>
-      <c r="L10" s="91" t="inlineStr">
+      <c r="E10" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L10" s="91" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1" s="60">
       <c r="A11" s="5" t="n"/>
@@ -2045,11 +2052,12 @@
           <t>Exploration mission list — reward typo fixed</t>
         </is>
       </c>
-      <c r="L11" s="91" t="inlineStr">
+      <c r="E11" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L11" s="91" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1" s="60">
       <c r="A12" s="5" t="n"/>
@@ -2066,11 +2074,12 @@
           <t>Stamina Potion reward removed</t>
         </is>
       </c>
-      <c r="L12" s="91" t="inlineStr">
+      <c r="E12" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L12" s="91" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1" s="60">
       <c r="A13" s="5" t="n"/>
@@ -2084,14 +2093,15 @@
       </c>
       <c r="D13" s="88" t="inlineStr">
         <is>
-          <t>Sage's Library exploration missions added</t>
-        </is>
-      </c>
-      <c r="L13" s="91" t="inlineStr">
+          <t>Library of Sage exploration missions added</t>
+        </is>
+      </c>
+      <c r="E13" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L13" s="91" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1" s="60">
       <c r="A14" s="5" t="n"/>
@@ -2105,14 +2115,15 @@
       </c>
       <c r="D14" s="88" t="inlineStr">
         <is>
-          <t>Sage's Library exploration mission rewards specified</t>
-        </is>
-      </c>
-      <c r="L14" s="91" t="inlineStr">
+          <t>Library of Sage exploration mission rewards specified</t>
+        </is>
+      </c>
+      <c r="E14" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L14" s="91" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1" s="60">
       <c r="A15" s="5" t="n"/>
@@ -2129,11 +2140,12 @@
           <t>Will-o'-Wisp defeat mission removed</t>
         </is>
       </c>
-      <c r="L15" s="91" t="inlineStr">
+      <c r="E15" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L15" s="91" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1" s="60">
       <c r="A16" s="5" t="n"/>
@@ -2150,11 +2162,12 @@
           <t>Difficult monster defeat exploration missions removed</t>
         </is>
       </c>
-      <c r="L16" s="91" t="inlineStr">
+      <c r="E16" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L16" s="91" t="n"/>
     </row>
     <row r="17" ht="18" customHeight="1" s="60">
       <c r="A17" s="5" t="n"/>
@@ -2171,11 +2184,12 @@
           <t>Completed reward areas greyed out in list</t>
         </is>
       </c>
-      <c r="L17" s="91" t="inlineStr">
+      <c r="E17" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L17" s="91" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1" s="60">
       <c r="A18" s="5" t="n"/>
@@ -2192,11 +2206,12 @@
           <t>Reward list updated</t>
         </is>
       </c>
-      <c r="L18" s="91" t="inlineStr">
+      <c r="E18" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L18" s="91" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1" s="60">
       <c r="A19" s="5" t="n"/>
@@ -2213,11 +2228,12 @@
           <t>Spring Waterway rewards modified</t>
         </is>
       </c>
-      <c r="L19" s="91" t="inlineStr">
+      <c r="E19" s="0" t="inlineStr">
         <is>
           <t>Juwon Lee</t>
         </is>
       </c>
+      <c r="L19" s="91" t="n"/>
     </row>
     <row r="20" ht="15.75" customHeight="1" s="60">
       <c r="A20" s="5" t="n"/>
@@ -5686,7 +5702,7 @@
       <c r="B98" s="25" t="n"/>
       <c r="C98" s="29" t="inlineStr">
         <is>
-          <t>→ Wind Valley, Submerged Passage Etc.</t>
+          <t>→ Windy Valley, Submerged Passage Etc.</t>
         </is>
       </c>
       <c r="D98" s="25" t="n"/>
@@ -14516,13 +14532,13 @@
     <row r="431" s="60">
       <c r="B431" s="58" t="inlineStr">
         <is>
-          <t>Silak's Mansion</t>
+          <t>Mansion of Syllek</t>
         </is>
       </c>
       <c r="C431" s="58" t="n"/>
       <c r="D431" s="58" t="inlineStr">
         <is>
-          <t>Silak's Mansion World</t>
+          <t>Mansion of Syllek World</t>
         </is>
       </c>
       <c r="E431" s="58" t="n">
@@ -14744,7 +14760,7 @@
       </c>
       <c r="D443" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Silak's Mansion </t>
+          <t xml:space="preserve">Mansion of Syllek </t>
         </is>
       </c>
       <c r="E443" s="58" t="n">
@@ -14800,7 +14816,7 @@
       </c>
       <c r="D446" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Silak's Mansion </t>
+          <t xml:space="preserve">Mansion of Syllek </t>
         </is>
       </c>
       <c r="E446" s="58" t="n">
@@ -15864,7 +15880,7 @@
       </c>
       <c r="D505" s="58" t="inlineStr">
         <is>
-          <t>Silak's Mansion Hunting Ground</t>
+          <t>Mansion of Syllek Hunting Ground</t>
         </is>
       </c>
       <c r="E505" s="58" t="n">
@@ -16744,7 +16760,7 @@
       </c>
       <c r="D554" s="58" t="inlineStr">
         <is>
-          <t>Silak's Mansion th Hunting Ground</t>
+          <t>Mansion of Syllek th Hunting Ground</t>
         </is>
       </c>
       <c r="E554" s="58" t="n">
@@ -17052,13 +17068,13 @@
     <row r="571" s="60">
       <c r="B571" s="58" t="inlineStr">
         <is>
-          <t>Wind Valley</t>
+          <t>Windy Valley</t>
         </is>
       </c>
       <c r="C571" s="58" t="n"/>
       <c r="D571" s="58" t="inlineStr">
         <is>
-          <t>Wind Valley World</t>
+          <t>Windy Valley World</t>
         </is>
       </c>
       <c r="E571" s="58" t="n">
@@ -17120,7 +17136,7 @@
       </c>
       <c r="D574" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wind Valley </t>
+          <t xml:space="preserve">Windy Valley </t>
         </is>
       </c>
       <c r="E574" s="58" t="n">
@@ -17160,7 +17176,7 @@
       </c>
       <c r="D576" s="58" t="inlineStr">
         <is>
-          <t>Wind Valley Deep Place</t>
+          <t>Windy Valley Deep Place</t>
         </is>
       </c>
       <c r="E576" s="58" t="n">
@@ -17212,13 +17228,13 @@
     <row r="579" s="60">
       <c r="B579" s="58" t="inlineStr">
         <is>
-          <t>Burning Furnace</t>
+          <t>Burning Forge</t>
         </is>
       </c>
       <c r="C579" s="58" t="n"/>
       <c r="D579" s="58" t="inlineStr">
         <is>
-          <t>Burning Furnace World</t>
+          <t>Burning Forge World</t>
         </is>
       </c>
       <c r="E579" s="58" t="n">
@@ -17344,7 +17360,7 @@
       </c>
       <c r="D586" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Burning Furnace </t>
+          <t xml:space="preserve">Burning Forge </t>
         </is>
       </c>
       <c r="E586" s="58" t="n">
@@ -18096,7 +18112,7 @@
       </c>
       <c r="D628" s="58" t="inlineStr">
         <is>
-          <t>Burning Furnace Hunting Ground</t>
+          <t>Burning Forge Hunting Ground</t>
         </is>
       </c>
       <c r="E628" s="58" t="n">
@@ -19016,7 +19032,7 @@
       </c>
       <c r="D680" s="58" t="inlineStr">
         <is>
-          <t>Burning Furnace th Hunting Ground</t>
+          <t>Burning Forge th Hunting Ground</t>
         </is>
       </c>
       <c r="E680" s="58" t="n">
@@ -19868,13 +19884,13 @@
     <row r="727" s="60">
       <c r="B727" s="58" t="inlineStr">
         <is>
-          <t>Sage's Library</t>
+          <t>Library of Sage</t>
         </is>
       </c>
       <c r="C727" s="58" t="n"/>
       <c r="D727" s="58" t="inlineStr">
         <is>
-          <t>Sage's Library World</t>
+          <t>Library of Sage World</t>
         </is>
       </c>
       <c r="E727" s="58" t="n">
@@ -20616,7 +20632,7 @@
       </c>
       <c r="D768" s="58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sage's Library </t>
+          <t xml:space="preserve">Library of Sage </t>
         </is>
       </c>
       <c r="E768" s="58" t="n">
@@ -20688,7 +20704,7 @@
       </c>
       <c r="D772" s="58" t="inlineStr">
         <is>
-          <t>Sage's Library Entrance</t>
+          <t>Library of Sage Entrance</t>
         </is>
       </c>
       <c r="E772" s="58" t="n">
@@ -21080,7 +21096,7 @@
       </c>
       <c r="D794" s="58" t="inlineStr">
         <is>
-          <t>Sage's Library Hunting Ground</t>
+          <t>Library of Sage Hunting Ground</t>
         </is>
       </c>
       <c r="E794" s="58" t="n">
@@ -22000,7 +22016,7 @@
       </c>
       <c r="D847" s="58" t="inlineStr">
         <is>
-          <t>Sage's Library th Hunting Ground</t>
+          <t>Library of Sage th Hunting Ground</t>
         </is>
       </c>
       <c r="E847" s="58" t="n">

</xml_diff>

<commit_message>
Rewrite Design Intent sections + fix data table patterns
- All 7 XLSX: Design Intent/Summary/Policy retranslated from Korean originals
- Exploration Missions: garbled text completely rewritten
- Dimensional Gate: "zone move" → proper fast-travel description
- Time Gate: "gimmick" → cinematic world-building explanation
- Quest Guide: table headers and special notes corrected
- Data tables: "10times" → "10×", "Grade/Tier" → "Grade" (170 cells)
- Author column width: E=18, L reset to default (6 files)

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/ExplorationMissions_DesignDocument.xlsx
+++ b/docs/ExplorationMissions_DesignDocument.xlsx
@@ -1831,7 +1831,8 @@
     <col width="8" customWidth="1" style="43" min="2" max="2"/>
     <col width="12" customWidth="1" style="43" min="3" max="3"/>
     <col width="75" customWidth="1" style="43" min="4" max="15"/>
-    <col width="18" customWidth="1" style="60" min="12" max="12"/>
+    <col width="18" customWidth="1" style="60" min="5" max="5"/>
+    <col width="8.43" customWidth="1" style="60" min="12" max="12"/>
     <col width="11.375" bestFit="1" customWidth="1" style="43" min="16" max="16"/>
     <col width="9" customWidth="1" style="43" min="17" max="16384"/>
   </cols>
@@ -2528,7 +2529,7 @@
       <c r="C7" s="15" t="n"/>
       <c r="D7" s="18" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>- Provides direction and goals for exploring every corner of the field</t>
         </is>
       </c>
       <c r="E7" s="15" t="n"/>
@@ -2565,7 +2566,7 @@
       <c r="C8" s="15" t="n"/>
       <c r="D8" s="18" t="inlineStr">
         <is>
-          <t>- PLC</t>
+          <t>- Grants PLC (player-lifecycle currency) and gameplay-essential resources</t>
         </is>
       </c>
       <c r="E8" s="15" t="n"/>
@@ -2704,7 +2705,7 @@
       <c r="B12" s="15" t="n"/>
       <c r="C12" s="23" t="inlineStr">
         <is>
-          <t>- Exploration Mission Exploration Mission zone Exploration Mission 2</t>
+          <t>- Exploration Missions are categorized into World-level and Area-level missions</t>
         </is>
       </c>
       <c r="D12" s="22" t="n"/>
@@ -2741,7 +2742,7 @@
       <c r="B13" s="15" t="n"/>
       <c r="C13" s="23" t="inlineStr">
         <is>
-          <t>- Exploration Mission Complete when, Reward Grant</t>
+          <t>- Rewards are granted upon mission completion</t>
         </is>
       </c>
       <c r="D13" s="22" t="n"/>
@@ -2778,7 +2779,7 @@
       <c r="B14" s="15" t="n"/>
       <c r="C14" s="23" t="inlineStr">
         <is>
-          <t>- Separate's Accept Always Progressduring state</t>
+          <t>- Missions are always in progress without requiring manual acceptance</t>
         </is>
       </c>
       <c r="D14" s="18" t="n"/>
@@ -2815,7 +2816,7 @@
       <c r="B15" s="15" t="n"/>
       <c r="C15" s="23" t="inlineStr">
         <is>
-          <t>- World and Area Provide</t>
+          <t>- Objectives reflect the unique characteristics of each world and area</t>
         </is>
       </c>
       <c r="D15" s="18" t="n"/>
@@ -6035,7 +6036,7 @@
       <c r="B107" s="25" t="n"/>
       <c r="C107" s="31" t="inlineStr">
         <is>
-          <t>- World Exploration Mission : List during Achieve when, All Achieve when 2times Reward</t>
+          <t>- World Exploration Mission : List during Achieve when, All Achieve when 2× Reward</t>
         </is>
       </c>
       <c r="D107" s="25" t="n"/>
@@ -6072,7 +6073,7 @@
       <c r="B108" s="25" t="n"/>
       <c r="C108" s="31" t="inlineStr">
         <is>
-          <t>- Area Exploration Mission : List before Achieve when, 1times Reward</t>
+          <t>- Area Exploration Mission : List before Achieve when, 1× Reward</t>
         </is>
       </c>
       <c r="D108" s="25" t="n"/>

</xml_diff>

<commit_message>
Remove IP protection: restore original images + data, keep CONFIDENTIAL on half world maps only
- Restored 366 images from pre-S18 backups (removed blur/watermark)
- Restored 1,058 masked numeric cells in Records
- Removed CONFIDENTIAL watermark overlays from all sheets
- Kept selective CONFIDENTIAL on ~50% of World overview maps (개형도)
- All S19 translation fixes preserved
</commit_message>
<xml_diff>
--- a/docs/ExplorationMissions_DesignDocument.xlsx
+++ b/docs/ExplorationMissions_DesignDocument.xlsx
@@ -1047,460 +1047,460 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>2</col>
-      <colOff>1</colOff>
-      <row>32</row>
-      <rowOff>28575</rowOff>
-    </from>
-    <to>
-      <col>36</col>
-      <colOff>9526</colOff>
-      <row>52</row>
-      <rowOff>92910</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="72" name="그림 71"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+<ns0:wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:ns0="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:ns2="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:twoCellAnchor editAs="oneCell">
+    <ns0:from>
+      <ns0:col>2</ns0:col>
+      <ns0:colOff>1</ns0:colOff>
+      <ns0:row>32</ns0:row>
+      <ns0:rowOff>28575</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>36</ns0:col>
+      <ns0:colOff>9526</ns0:colOff>
+      <ns0:row>52</ns0:row>
+      <ns0:rowOff>92910</ns0:rowOff>
+    </ns0:to>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="72" name="그림 71"/>
+        <ns0:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <a:blip ns2:embed="rId1"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:blipFill>
+      <ns0:spPr>
+        <a:xfrm>
           <a:off x="400051" y="6734175"/>
           <a:ext cx="7600950" cy="4255335"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
+        <a:prstGeom prst="rect">
+          <ns0:avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>188965</colOff>
-      <row>55</row>
-      <rowOff>114354</rowOff>
-    </from>
-    <to>
-      <col>40</col>
-      <colOff>30418</colOff>
-      <row>77</row>
-      <rowOff>142820</rowOff>
-    </to>
-    <grpSp>
-      <nvGrpSpPr>
-        <cNvPr id="73" name="그룹 72"/>
-        <cNvGrpSpPr/>
-      </nvGrpSpPr>
-      <grpSpPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor>
+    <ns0:from>
+      <ns0:col>0</ns0:col>
+      <ns0:colOff>188965</ns0:colOff>
+      <ns0:row>55</ns0:row>
+      <ns0:rowOff>114354</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>40</ns0:col>
+      <ns0:colOff>30418</ns0:colOff>
+      <ns0:row>77</ns0:row>
+      <ns0:rowOff>142820</ns0:rowOff>
+    </ns0:to>
+    <ns0:grpSp>
+      <ns0:nvGrpSpPr>
+        <ns0:cNvPr id="73" name="그룹 72"/>
+        <ns0:cNvGrpSpPr/>
+      </ns0:nvGrpSpPr>
+      <ns0:grpSpPr>
+        <a:xfrm rot="0">
           <a:off x="188965" y="11639604"/>
           <a:ext cx="8633028" cy="4638566"/>
           <a:chOff x="-271771" y="33337"/>
           <a:chExt cx="12430433" cy="6791325"/>
         </a:xfrm>
-      </grpSpPr>
-      <pic>
-        <nvPicPr>
-          <cNvPr id="76" name="그림 75"/>
-          <cNvPicPr>
-            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-          </cNvPicPr>
-        </nvPicPr>
-        <blipFill>
-          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
-          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:grpSpPr>
+      <ns0:pic>
+        <ns0:nvPicPr>
+          <ns0:cNvPr id="76" name="그림 75"/>
+          <ns0:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </ns0:cNvPicPr>
+        </ns0:nvPicPr>
+        <ns0:blipFill>
+          <a:blip ns2:embed="rId2"/>
+          <a:stretch>
             <a:fillRect/>
           </a:stretch>
-        </blipFill>
-        <spPr>
-          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        </ns0:blipFill>
+        <ns0:spPr>
+          <a:xfrm>
             <a:off x="3743880" y="101122"/>
             <a:ext cx="3905250" cy="1400175"/>
           </a:xfrm>
-          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-            <avLst/>
+          <a:prstGeom prst="rect">
+            <ns0:avLst/>
           </a:prstGeom>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:ln>
             <a:prstDash val="solid"/>
           </a:ln>
-        </spPr>
-      </pic>
-    </grpSp>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>12</col>
-      <colOff>9526</colOff>
-      <row>85</row>
-      <rowOff>2990850</rowOff>
-    </from>
-    <to>
-      <col>14</col>
-      <colOff>24164</colOff>
-      <row>85</row>
-      <rowOff>3438525</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="96" name="그림 95"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        </ns0:spPr>
+      </ns0:pic>
+    </ns0:grpSp>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor editAs="oneCell">
+    <ns0:from>
+      <ns0:col>12</ns0:col>
+      <ns0:colOff>9526</ns0:colOff>
+      <ns0:row>85</ns0:row>
+      <ns0:rowOff>2990850</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>14</ns0:col>
+      <ns0:colOff>24164</ns0:colOff>
+      <ns0:row>85</ns0:row>
+      <ns0:rowOff>3438525</ns0:rowOff>
+    </ns0:to>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="96" name="그림 95"/>
+        <ns0:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <a:blip ns2:embed="rId3"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:blipFill>
+      <ns0:spPr>
+        <a:xfrm>
           <a:off x="3057526" y="27470100"/>
           <a:ext cx="414688" cy="447675"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
+        <a:prstGeom prst="rect">
+          <ns0:avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>12</col>
-      <colOff>28575</colOff>
-      <row>85</row>
-      <rowOff>3838575</rowOff>
-    </from>
-    <to>
-      <col>14</col>
-      <colOff>68929</colOff>
-      <row>85</row>
-      <rowOff>4314825</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="97" name="그림 96"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId4"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor editAs="oneCell">
+    <ns0:from>
+      <ns0:col>12</ns0:col>
+      <ns0:colOff>28575</ns0:colOff>
+      <ns0:row>85</ns0:row>
+      <ns0:rowOff>3838575</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>14</ns0:col>
+      <ns0:colOff>68929</ns0:colOff>
+      <ns0:row>85</ns0:row>
+      <ns0:rowOff>4314825</ns0:rowOff>
+    </ns0:to>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="97" name="그림 96"/>
+        <ns0:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <a:blip ns2:embed="rId4"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:blipFill>
+      <ns0:spPr>
+        <a:xfrm>
           <a:off x="3076575" y="28317825"/>
           <a:ext cx="440404" cy="476250"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
+        <a:prstGeom prst="rect">
+          <ns0:avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>12</col>
-      <colOff>28575</colOff>
-      <row>85</row>
-      <rowOff>4695825</rowOff>
-    </from>
-    <to>
-      <col>14</col>
-      <colOff>68904</colOff>
-      <row>86</row>
-      <rowOff>0</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="98" name="그림 97"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor editAs="oneCell">
+    <ns0:from>
+      <ns0:col>12</ns0:col>
+      <ns0:colOff>28575</ns0:colOff>
+      <ns0:row>85</ns0:row>
+      <ns0:rowOff>4695825</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>14</ns0:col>
+      <ns0:colOff>68904</ns0:colOff>
+      <ns0:row>86</ns0:row>
+      <ns0:rowOff>0</ns0:rowOff>
+    </ns0:to>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="98" name="그림 97"/>
+        <ns0:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <a:blip ns2:embed="rId5"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:blipFill>
+      <ns0:spPr>
+        <a:xfrm>
           <a:off x="3076575" y="29832300"/>
           <a:ext cx="440379" cy="504825"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
+        <a:prstGeom prst="rect">
+          <ns0:avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>10</col>
-      <colOff>95250</colOff>
-      <row>80</row>
-      <rowOff>1971675</rowOff>
-    </from>
-    <to>
-      <col>12</col>
-      <colOff>133295</colOff>
-      <row>80</row>
-      <rowOff>2400246</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="99" name="그림 98"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId6"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor editAs="oneCell">
+    <ns0:from>
+      <ns0:col>10</ns0:col>
+      <ns0:colOff>95250</ns0:colOff>
+      <ns0:row>80</ns0:row>
+      <ns0:rowOff>1971675</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>12</ns0:col>
+      <ns0:colOff>133295</ns0:colOff>
+      <ns0:row>80</ns0:row>
+      <ns0:rowOff>2400246</ns0:rowOff>
+    </ns0:to>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="99" name="그림 98"/>
+        <ns0:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <a:blip ns2:embed="rId6"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:blipFill>
+      <ns0:spPr>
+        <a:xfrm>
           <a:off x="2743200" y="19554825"/>
           <a:ext cx="438095" cy="428571"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
+        <a:prstGeom prst="rect">
+          <ns0:avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>10</col>
-      <colOff>85725</colOff>
-      <row>80</row>
-      <rowOff>1114192</rowOff>
-    </from>
-    <to>
-      <col>12</col>
-      <colOff>133350</colOff>
-      <row>80</row>
-      <rowOff>1485847</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="100" name="그림 99"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor editAs="oneCell">
+    <ns0:from>
+      <ns0:col>10</ns0:col>
+      <ns0:colOff>85725</ns0:colOff>
+      <ns0:row>80</ns0:row>
+      <ns0:rowOff>1114192</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>12</ns0:col>
+      <ns0:colOff>133350</ns0:colOff>
+      <ns0:row>80</ns0:row>
+      <ns0:rowOff>1485847</ns0:rowOff>
+    </ns0:to>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="100" name="그림 99"/>
+        <ns0:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <a:blip ns2:embed="rId7"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:blipFill>
+      <ns0:spPr>
+        <a:xfrm>
           <a:off x="2733675" y="18697342"/>
           <a:ext cx="447675" cy="371655"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
+        <a:prstGeom prst="rect">
+          <ns0:avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor>
-    <from>
-      <col>1</col>
-      <colOff>65699</colOff>
-      <row>113</row>
-      <rowOff>75339</rowOff>
-    </from>
-    <to>
-      <col>40</col>
-      <colOff>27134</colOff>
-      <row>129</row>
-      <rowOff>34844</rowOff>
-    </to>
-    <grpSp>
-      <nvGrpSpPr>
-        <cNvPr id="101" name="그룹 100"/>
-        <cNvGrpSpPr/>
-      </nvGrpSpPr>
-      <grpSpPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor>
+    <ns0:from>
+      <ns0:col>1</ns0:col>
+      <ns0:colOff>65699</ns0:colOff>
+      <ns0:row>113</ns0:row>
+      <ns0:rowOff>75339</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>40</ns0:col>
+      <ns0:colOff>27134</ns0:colOff>
+      <ns0:row>129</ns0:row>
+      <ns0:rowOff>34844</ns0:rowOff>
+    </ns0:to>
+    <ns0:grpSp>
+      <ns0:nvGrpSpPr>
+        <ns0:cNvPr id="101" name="그룹 100"/>
+        <ns0:cNvGrpSpPr/>
+      </ns0:nvGrpSpPr>
+      <ns0:grpSpPr>
+        <a:xfrm rot="0">
           <a:off x="265724" y="40004139"/>
           <a:ext cx="8552985" cy="2702705"/>
           <a:chOff x="-18662" y="1043233"/>
           <a:chExt cx="24402662" cy="7711132"/>
         </a:xfrm>
-      </grpSpPr>
-      <pic>
-        <nvPicPr>
-          <cNvPr id="105" name="그림 104"/>
-          <cNvPicPr>
-            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-          </cNvPicPr>
-        </nvPicPr>
-        <blipFill>
-          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8"/>
-          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:grpSpPr>
+      <ns0:pic>
+        <ns0:nvPicPr>
+          <ns0:cNvPr id="105" name="그림 104"/>
+          <ns0:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </ns0:cNvPicPr>
+        </ns0:nvPicPr>
+        <ns0:blipFill>
+          <a:blip ns2:embed="rId8"/>
+          <a:stretch>
             <a:fillRect/>
           </a:stretch>
-        </blipFill>
-        <spPr>
-          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        </ns0:blipFill>
+        <ns0:spPr>
+          <a:xfrm>
             <a:off x="12192000" y="5637484"/>
             <a:ext cx="12192000" cy="3116880"/>
           </a:xfrm>
-          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-            <avLst/>
+          <a:prstGeom prst="rect">
+            <ns0:avLst/>
           </a:prstGeom>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:ln>
             <a:prstDash val="solid"/>
           </a:ln>
-        </spPr>
-      </pic>
-    </grpSp>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>23</col>
-      <colOff>9525</colOff>
-      <row>81</row>
-      <rowOff>3143250</rowOff>
-    </from>
-    <to>
-      <col>29</col>
-      <colOff>152232</colOff>
-      <row>81</row>
-      <rowOff>3467060</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="그림 1"/>
-        <cNvPicPr>
-          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-        </cNvPicPr>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        </ns0:spPr>
+      </ns0:pic>
+    </ns0:grpSp>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor editAs="oneCell">
+    <ns0:from>
+      <ns0:col>23</ns0:col>
+      <ns0:colOff>9525</ns0:colOff>
+      <ns0:row>81</ns0:row>
+      <ns0:rowOff>3143250</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>29</ns0:col>
+      <ns0:colOff>152232</ns0:colOff>
+      <ns0:row>81</ns0:row>
+      <ns0:rowOff>3467060</ns0:rowOff>
+    </ns0:to>
+    <ns0:pic>
+      <ns0:nvPicPr>
+        <ns0:cNvPr id="2" name="그림 1"/>
+        <ns0:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </ns0:cNvPicPr>
+      </ns0:nvPicPr>
+      <ns0:blipFill>
+        <a:blip ns2:embed="rId9"/>
+        <a:stretch>
           <a:fillRect/>
         </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:blipFill>
+      <ns0:spPr>
+        <a:xfrm>
           <a:off x="5400675" y="23860125"/>
           <a:ext cx="1342857" cy="323810"/>
         </a:xfrm>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-          <avLst/>
+        <a:prstGeom prst="rect">
+          <ns0:avLst/>
         </a:prstGeom>
-        <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:ln>
           <a:prstDash val="solid"/>
         </a:ln>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>20</row>
-      <rowOff>0</rowOff>
-    </from>
-    <to>
-      <col>43</col>
-      <colOff>2293</colOff>
-      <row>30</row>
-      <rowOff>74718</rowOff>
-    </to>
-    <grpSp>
-      <nvGrpSpPr>
-        <cNvPr id="3" name="그룹 2"/>
-        <cNvGrpSpPr/>
-      </nvGrpSpPr>
-      <grpSpPr>
-        <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" rot="0">
+      </ns0:spPr>
+    </ns0:pic>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+  <ns0:twoCellAnchor>
+    <ns0:from>
+      <ns0:col>2</ns0:col>
+      <ns0:colOff>0</ns0:colOff>
+      <ns0:row>20</ns0:row>
+      <ns0:rowOff>0</ns0:rowOff>
+    </ns0:from>
+    <ns0:to>
+      <ns0:col>43</ns0:col>
+      <ns0:colOff>2293</ns0:colOff>
+      <ns0:row>30</ns0:row>
+      <ns0:rowOff>74718</ns0:rowOff>
+    </ns0:to>
+    <ns0:grpSp>
+      <ns0:nvGrpSpPr>
+        <ns0:cNvPr id="3" name="그룹 2"/>
+        <ns0:cNvGrpSpPr/>
+      </ns0:nvGrpSpPr>
+      <ns0:grpSpPr>
+        <a:xfrm rot="0">
           <a:off x="400050" y="4191000"/>
           <a:ext cx="8993893" cy="2170218"/>
           <a:chOff x="-1605579" y="3199191"/>
           <a:chExt cx="13167958" cy="3177416"/>
         </a:xfrm>
-      </grpSpPr>
-      <pic>
-        <nvPicPr>
-          <cNvPr id="5" name="그림 4"/>
-          <cNvPicPr>
-            <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
-          </cNvPicPr>
-        </nvPicPr>
-        <blipFill>
-          <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10"/>
-          <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      </ns0:grpSpPr>
+      <ns0:pic>
+        <ns0:nvPicPr>
+          <ns0:cNvPr id="5" name="그림 4"/>
+          <ns0:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </ns0:cNvPicPr>
+        </ns0:nvPicPr>
+        <ns0:blipFill>
+          <a:blip ns2:embed="rId10"/>
+          <a:stretch>
             <a:fillRect/>
           </a:stretch>
-        </blipFill>
-        <spPr>
-          <a:xfrm xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        </ns0:blipFill>
+        <ns0:spPr>
+          <a:xfrm>
             <a:off x="5874721" y="3199191"/>
             <a:ext cx="5687658" cy="3174987"/>
           </a:xfrm>
-          <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
-            <avLst/>
+          <a:prstGeom prst="rect">
+            <ns0:avLst/>
           </a:prstGeom>
-          <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:ln>
             <a:prstDash val="solid"/>
           </a:ln>
-        </spPr>
-      </pic>
-    </grpSp>
-    <clientData/>
-  </twoCellAnchor>
-</wsDr>
+        </ns0:spPr>
+      </ns0:pic>
+    </ns0:grpSp>
+    <ns0:clientData/>
+  </ns0:twoCellAnchor>
+</ns0:wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>